<commit_message>
Petite Cup 48 (S3 R19): ZOMAN back-to-back, Lexer Curse FFF
- Finals: ZOMAN 20.938 over justMaki 21.007 (~69ms) — ZOMAN takes
  consecutive PCDJ wins after dethroning Maki's streak in cup 47
- Eclipse135 3rd (R12), Lexer 4th by DNF (R11) — the Curse continues
- 25 ranked: [Buny]Lunarbunny excluded as map 2 mapper; PlusMicron
  sat out as map 1 mapper
- Maps: PCDJ #48 - Manjaro by PlusMicron + Mountain pass by Luna
- aizpun couldn't play; standings reconstructed from justMaki's VOD
  (no local COTDTracker/LiveLeaderboardLogger logs for this cup)
- status.json reset to post-Cup-47 baseline (prior snapshot was
  post-Cup-46; cup 47 was committed without a pre-snapshot, so arrows
  would have shown 2 rounds of change otherwise)
</commit_message>
<xml_diff>
--- a/Petite Cups 46-50.xlsx
+++ b/Petite Cups 46-50.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:J44"/>
+  <dimension ref="A2:P59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="2">
@@ -427,6 +427,11 @@
           <t>Petite Cup 47</t>
         </is>
       </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>Petite Cup 48</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -439,6 +444,11 @@
           <t>Maps: PCDJ 47 - Neone + PCDJ 47 - Home Sweet Hole</t>
         </is>
       </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>Maps: PCDJ #48 - Manjaro by PlusMicron + PCDJ #48 - Mountain pass by Luna</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -477,6 +487,26 @@
         </is>
       </c>
       <c r="J5" t="inlineStr">
+        <is>
+          <t>Elim Round</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>Position</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>Elim Time</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
         <is>
           <t>Elim Round</t>
         </is>
@@ -505,6 +535,17 @@
       <c r="I6" t="n">
         <v>24.02438</v>
       </c>
+      <c r="M6" t="n">
+        <v>1</v>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>ZOMAN</t>
+        </is>
+      </c>
+      <c r="O6" t="n">
+        <v>20.938</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -535,6 +576,20 @@
       <c r="J7" t="n">
         <v>13</v>
       </c>
+      <c r="M7" t="n">
+        <v>2</v>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>justMaki</t>
+        </is>
+      </c>
+      <c r="O7" t="n">
+        <v>21.007</v>
+      </c>
+      <c r="P7" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -565,6 +620,20 @@
       <c r="J8" t="n">
         <v>12</v>
       </c>
+      <c r="M8" t="n">
+        <v>3</v>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>Eclipse135</t>
+        </is>
+      </c>
+      <c r="O8" t="n">
+        <v>18.629</v>
+      </c>
+      <c r="P8" t="n">
+        <v>12</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -597,6 +666,22 @@
       <c r="J9" t="n">
         <v>11</v>
       </c>
+      <c r="M9" t="n">
+        <v>4</v>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>Lexer</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>DNF</t>
+        </is>
+      </c>
+      <c r="P9" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -627,6 +712,22 @@
       <c r="J10" t="n">
         <v>10</v>
       </c>
+      <c r="M10" t="n">
+        <v>5</v>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>Mμ</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>DNF</t>
+        </is>
+      </c>
+      <c r="P10" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -657,6 +758,20 @@
       <c r="J11" t="n">
         <v>9</v>
       </c>
+      <c r="M11" t="n">
+        <v>6</v>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>ping</t>
+        </is>
+      </c>
+      <c r="O11" t="n">
+        <v>21.24479</v>
+      </c>
+      <c r="P11" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -687,6 +802,20 @@
       <c r="J12" t="n">
         <v>8</v>
       </c>
+      <c r="M12" t="n">
+        <v>7</v>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>[CSC]Tommygaming</t>
+        </is>
+      </c>
+      <c r="O12" t="n">
+        <v>18.75155</v>
+      </c>
+      <c r="P12" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -719,6 +848,20 @@
       <c r="J13" t="n">
         <v>8</v>
       </c>
+      <c r="M13" t="n">
+        <v>8</v>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>Noxitu</t>
+        </is>
+      </c>
+      <c r="O13" t="n">
+        <v>18.77549</v>
+      </c>
+      <c r="P13" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -749,6 +892,20 @@
       <c r="J14" t="n">
         <v>7</v>
       </c>
+      <c r="M14" t="n">
+        <v>9</v>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>Matic_D</t>
+        </is>
+      </c>
+      <c r="O14" t="n">
+        <v>21.54511</v>
+      </c>
+      <c r="P14" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -779,6 +936,22 @@
       <c r="J15" t="n">
         <v>7</v>
       </c>
+      <c r="M15" t="n">
+        <v>10</v>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>icRS</t>
+        </is>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>DNF</t>
+        </is>
+      </c>
+      <c r="P15" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -809,6 +982,20 @@
       <c r="J16" t="n">
         <v>6</v>
       </c>
+      <c r="M16" t="n">
+        <v>11</v>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>racemaniac</t>
+        </is>
+      </c>
+      <c r="O16" t="n">
+        <v>18.87401</v>
+      </c>
+      <c r="P16" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -839,6 +1026,20 @@
       <c r="J17" t="n">
         <v>6</v>
       </c>
+      <c r="M17" t="n">
+        <v>12</v>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>[EEN] Hang Chang-Pang</t>
+        </is>
+      </c>
+      <c r="O17" t="n">
+        <v>18.88763</v>
+      </c>
+      <c r="P17" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -869,6 +1070,20 @@
       <c r="J18" t="n">
         <v>5</v>
       </c>
+      <c r="M18" t="n">
+        <v>13</v>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>Six</t>
+        </is>
+      </c>
+      <c r="O18" t="n">
+        <v>21.75123</v>
+      </c>
+      <c r="P18" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -899,6 +1114,20 @@
       <c r="J19" t="n">
         <v>5</v>
       </c>
+      <c r="M19" t="n">
+        <v>14</v>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>[Fenn]Lilly Fenn</t>
+        </is>
+      </c>
+      <c r="O19" t="n">
+        <v>21.82034</v>
+      </c>
+      <c r="P19" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -929,6 +1158,20 @@
       <c r="J20" t="n">
         <v>5</v>
       </c>
+      <c r="M20" t="n">
+        <v>15</v>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>Tudge Boat</t>
+        </is>
+      </c>
+      <c r="O20" t="n">
+        <v>18.95383</v>
+      </c>
+      <c r="P20" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -961,6 +1204,20 @@
       <c r="J21" t="n">
         <v>4</v>
       </c>
+      <c r="M21" t="n">
+        <v>16</v>
+      </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>[20x]K410K3N</t>
+        </is>
+      </c>
+      <c r="O21" t="n">
+        <v>19.00928</v>
+      </c>
+      <c r="P21" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -993,6 +1250,20 @@
       <c r="J22" t="n">
         <v>4</v>
       </c>
+      <c r="M22" t="n">
+        <v>17</v>
+      </c>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>Jorts</t>
+        </is>
+      </c>
+      <c r="O22" t="n">
+        <v>19.198</v>
+      </c>
+      <c r="P22" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -1025,6 +1296,20 @@
       <c r="J23" t="n">
         <v>4</v>
       </c>
+      <c r="M23" t="n">
+        <v>18</v>
+      </c>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>[MIB]Joe Beidl</t>
+        </is>
+      </c>
+      <c r="O23" t="n">
+        <v>22.053</v>
+      </c>
+      <c r="P23" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -1057,6 +1342,20 @@
       <c r="J24" t="n">
         <v>4</v>
       </c>
+      <c r="M24" t="n">
+        <v>19</v>
+      </c>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>timesprout</t>
+        </is>
+      </c>
+      <c r="O24" t="n">
+        <v>22.082</v>
+      </c>
+      <c r="P24" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -1089,6 +1388,20 @@
       <c r="J25" t="n">
         <v>4</v>
       </c>
+      <c r="M25" t="n">
+        <v>20</v>
+      </c>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>Ooohbilly</t>
+        </is>
+      </c>
+      <c r="O25" t="n">
+        <v>22.111</v>
+      </c>
+      <c r="P25" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -1121,6 +1434,20 @@
       <c r="J26" t="n">
         <v>4</v>
       </c>
+      <c r="M26" t="n">
+        <v>21</v>
+      </c>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>M4DSCOTSM4N</t>
+        </is>
+      </c>
+      <c r="O26" t="n">
+        <v>19.2759</v>
+      </c>
+      <c r="P26" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -1151,6 +1478,20 @@
       <c r="J27" t="n">
         <v>3</v>
       </c>
+      <c r="M27" t="n">
+        <v>22</v>
+      </c>
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>imagineaclevernamehere</t>
+        </is>
+      </c>
+      <c r="O27" t="n">
+        <v>19.79578</v>
+      </c>
+      <c r="P27" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -1183,6 +1524,20 @@
       <c r="J28" t="n">
         <v>3</v>
       </c>
+      <c r="M28" t="n">
+        <v>23</v>
+      </c>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>Telion</t>
+        </is>
+      </c>
+      <c r="O28" t="n">
+        <v>20.25833</v>
+      </c>
+      <c r="P28" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -1217,6 +1572,20 @@
       <c r="J29" t="n">
         <v>3</v>
       </c>
+      <c r="M29" t="n">
+        <v>24</v>
+      </c>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>[CCC]Shinikage221</t>
+        </is>
+      </c>
+      <c r="O29" t="n">
+        <v>23.07496</v>
+      </c>
+      <c r="P29" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -1247,6 +1616,20 @@
       <c r="J30" t="n">
         <v>2</v>
       </c>
+      <c r="M30" t="n">
+        <v>25</v>
+      </c>
+      <c r="N30" t="inlineStr">
+        <is>
+          <t>taagern</t>
+        </is>
+      </c>
+      <c r="O30" t="n">
+        <v>24.74876</v>
+      </c>
+      <c r="P30" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -1568,6 +1951,21 @@
         <v>1</v>
       </c>
     </row>
+    <row r="45"/>
+    <row r="46"/>
+    <row r="47"/>
+    <row r="48"/>
+    <row r="49"/>
+    <row r="50"/>
+    <row r="51"/>
+    <row r="52"/>
+    <row r="53"/>
+    <row r="54"/>
+    <row r="55"/>
+    <row r="56"/>
+    <row r="57"/>
+    <row r="58"/>
+    <row r="59"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Petite Cup 49 (S3 R20): justMaki wins, Lexer breaks the Curse
- Maki dominates the final on 425nm: 19.861 over Lexer 20.123
- Lexer takes SILVER (not 4th!) — first non-4th petite finish in ages,
  ending his Lexer Curse streak in dramatic fashion
- Sandals 3rd, Eclipse135 4th (another deep run), JakeAdjacent 5th
- SOF 92.8% — strongest petite of the season
- 35 ranked (36-player lobby; Mμ excluded as 425nm mapper;
  [Burp]Weak_Knees mapped Astral Smoothie but didn't play)
- Maps: PCDJ #49 - 425nm by Mμ + Astral Smoothie by [Burp]Weak_Knees
- aizpun finished 18th (R7 eliminated at 21.86332 on map 1)
- Parsed cleanly from local logs (no DNF overrides needed)
</commit_message>
<xml_diff>
--- a/Petite Cups 46-50.xlsx
+++ b/Petite Cups 46-50.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:P59"/>
+  <dimension ref="A2:V59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="2">
@@ -432,6 +432,11 @@
           <t>Petite Cup 48</t>
         </is>
       </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>Petite Cup 49</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -449,6 +454,11 @@
           <t>Maps: PCDJ #48 - Manjaro by PlusMicron + PCDJ #48 - Mountain pass by Luna</t>
         </is>
       </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>Maps: PCDJ #49 - 425nm by Mμ + PCDJ #49 - Astral Smoothie by [Burp]Weak_Knees</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -507,6 +517,26 @@
         </is>
       </c>
       <c r="P5" t="inlineStr">
+        <is>
+          <t>Elim Round</t>
+        </is>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>Position</t>
+        </is>
+      </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>Elim Time</t>
+        </is>
+      </c>
+      <c r="V5" t="inlineStr">
         <is>
           <t>Elim Round</t>
         </is>
@@ -546,6 +576,17 @@
       <c r="O6" t="n">
         <v>20.938</v>
       </c>
+      <c r="S6" t="n">
+        <v>1</v>
+      </c>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>justMaki</t>
+        </is>
+      </c>
+      <c r="U6" t="n">
+        <v>19.86089</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -590,6 +631,20 @@
       <c r="P7" t="n">
         <v>13</v>
       </c>
+      <c r="S7" t="n">
+        <v>2</v>
+      </c>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>Lexer</t>
+        </is>
+      </c>
+      <c r="U7" t="n">
+        <v>20.12283</v>
+      </c>
+      <c r="V7" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -634,6 +689,20 @@
       <c r="P8" t="n">
         <v>12</v>
       </c>
+      <c r="S8" t="n">
+        <v>3</v>
+      </c>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t>[CTR] Sandals</t>
+        </is>
+      </c>
+      <c r="U8" t="n">
+        <v>21.09593</v>
+      </c>
+      <c r="V8" t="n">
+        <v>15</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -682,6 +751,20 @@
       <c r="P9" t="n">
         <v>11</v>
       </c>
+      <c r="S9" t="n">
+        <v>4</v>
+      </c>
+      <c r="T9" t="inlineStr">
+        <is>
+          <t>Eclipse135</t>
+        </is>
+      </c>
+      <c r="U9" t="n">
+        <v>20.43733</v>
+      </c>
+      <c r="V9" t="n">
+        <v>14</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -728,6 +811,20 @@
       <c r="P10" t="n">
         <v>10</v>
       </c>
+      <c r="S10" t="n">
+        <v>5</v>
+      </c>
+      <c r="T10" t="inlineStr">
+        <is>
+          <t>JakeAdjacent</t>
+        </is>
+      </c>
+      <c r="U10" t="n">
+        <v>21.22449</v>
+      </c>
+      <c r="V10" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -772,6 +869,20 @@
       <c r="P11" t="n">
         <v>9</v>
       </c>
+      <c r="S11" t="n">
+        <v>6</v>
+      </c>
+      <c r="T11" t="inlineStr">
+        <is>
+          <t>[KURK] Quickracer10</t>
+        </is>
+      </c>
+      <c r="U11" t="n">
+        <v>20.19603</v>
+      </c>
+      <c r="V11" t="n">
+        <v>12</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -816,6 +927,20 @@
       <c r="P12" t="n">
         <v>8</v>
       </c>
+      <c r="S12" t="n">
+        <v>7</v>
+      </c>
+      <c r="T12" t="inlineStr">
+        <is>
+          <t>[CSC]Tommygaming</t>
+        </is>
+      </c>
+      <c r="U12" t="n">
+        <v>21.37251</v>
+      </c>
+      <c r="V12" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -862,6 +987,22 @@
       <c r="P13" t="n">
         <v>8</v>
       </c>
+      <c r="S13" t="n">
+        <v>8</v>
+      </c>
+      <c r="T13" t="inlineStr">
+        <is>
+          <t>Shattersmith</t>
+        </is>
+      </c>
+      <c r="U13" t="inlineStr">
+        <is>
+          <t>DNF</t>
+        </is>
+      </c>
+      <c r="V13" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -906,6 +1047,20 @@
       <c r="P14" t="n">
         <v>7</v>
       </c>
+      <c r="S14" t="n">
+        <v>9</v>
+      </c>
+      <c r="T14" t="inlineStr">
+        <is>
+          <t>[CSC]AndMe17</t>
+        </is>
+      </c>
+      <c r="U14" t="n">
+        <v>20.24029</v>
+      </c>
+      <c r="V14" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -952,6 +1107,20 @@
       <c r="P15" t="n">
         <v>7</v>
       </c>
+      <c r="S15" t="n">
+        <v>10</v>
+      </c>
+      <c r="T15" t="inlineStr">
+        <is>
+          <t>𝒱V𝑜o𝒾i𝒹d𝒱</t>
+        </is>
+      </c>
+      <c r="U15" t="n">
+        <v>20.27772</v>
+      </c>
+      <c r="V15" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -996,6 +1165,20 @@
       <c r="P16" t="n">
         <v>6</v>
       </c>
+      <c r="S16" t="n">
+        <v>11</v>
+      </c>
+      <c r="T16" t="inlineStr">
+        <is>
+          <t>Diabler</t>
+        </is>
+      </c>
+      <c r="U16" t="n">
+        <v>21.40112</v>
+      </c>
+      <c r="V16" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -1040,6 +1223,20 @@
       <c r="P17" t="n">
         <v>6</v>
       </c>
+      <c r="S17" t="n">
+        <v>12</v>
+      </c>
+      <c r="T17" t="inlineStr">
+        <is>
+          <t>Hi Im Yolo</t>
+        </is>
+      </c>
+      <c r="U17" t="n">
+        <v>21.58975</v>
+      </c>
+      <c r="V17" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -1084,6 +1281,20 @@
       <c r="P18" t="n">
         <v>5</v>
       </c>
+      <c r="S18" t="n">
+        <v>13</v>
+      </c>
+      <c r="T18" t="inlineStr">
+        <is>
+          <t>RoundNzt</t>
+        </is>
+      </c>
+      <c r="U18" t="n">
+        <v>20.78679</v>
+      </c>
+      <c r="V18" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -1128,6 +1339,20 @@
       <c r="P19" t="n">
         <v>5</v>
       </c>
+      <c r="S19" t="n">
+        <v>14</v>
+      </c>
+      <c r="T19" t="inlineStr">
+        <is>
+          <t>brrryy</t>
+        </is>
+      </c>
+      <c r="U19" t="n">
+        <v>20.88211</v>
+      </c>
+      <c r="V19" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -1172,6 +1397,20 @@
       <c r="P20" t="n">
         <v>4</v>
       </c>
+      <c r="S20" t="n">
+        <v>15</v>
+      </c>
+      <c r="T20" t="inlineStr">
+        <is>
+          <t>Minkus</t>
+        </is>
+      </c>
+      <c r="U20" t="n">
+        <v>20.91721</v>
+      </c>
+      <c r="V20" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -1218,6 +1457,20 @@
       <c r="P21" t="n">
         <v>4</v>
       </c>
+      <c r="S21" t="n">
+        <v>16</v>
+      </c>
+      <c r="T21" t="inlineStr">
+        <is>
+          <t>ping</t>
+        </is>
+      </c>
+      <c r="U21" t="n">
+        <v>21.53531</v>
+      </c>
+      <c r="V21" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -1264,6 +1517,20 @@
       <c r="P22" t="n">
         <v>4</v>
       </c>
+      <c r="S22" t="n">
+        <v>17</v>
+      </c>
+      <c r="T22" t="inlineStr">
+        <is>
+          <t>Six</t>
+        </is>
+      </c>
+      <c r="U22" t="n">
+        <v>21.58115</v>
+      </c>
+      <c r="V22" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -1310,6 +1577,20 @@
       <c r="P23" t="n">
         <v>3</v>
       </c>
+      <c r="S23" t="n">
+        <v>18</v>
+      </c>
+      <c r="T23" t="inlineStr">
+        <is>
+          <t>aizpun</t>
+        </is>
+      </c>
+      <c r="U23" t="n">
+        <v>21.86332</v>
+      </c>
+      <c r="V23" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -1356,6 +1637,20 @@
       <c r="P24" t="n">
         <v>3</v>
       </c>
+      <c r="S24" t="n">
+        <v>19</v>
+      </c>
+      <c r="T24" t="inlineStr">
+        <is>
+          <t>Matic_D</t>
+        </is>
+      </c>
+      <c r="U24" t="n">
+        <v>21.22798</v>
+      </c>
+      <c r="V24" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -1402,6 +1697,20 @@
       <c r="P25" t="n">
         <v>3</v>
       </c>
+      <c r="S25" t="n">
+        <v>20</v>
+      </c>
+      <c r="T25" t="inlineStr">
+        <is>
+          <t>[ERR]ferinine</t>
+        </is>
+      </c>
+      <c r="U25" t="n">
+        <v>21.39687</v>
+      </c>
+      <c r="V25" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -1448,6 +1757,22 @@
       <c r="P26" t="n">
         <v>2</v>
       </c>
+      <c r="S26" t="n">
+        <v>21</v>
+      </c>
+      <c r="T26" t="inlineStr">
+        <is>
+          <t>Warsnac</t>
+        </is>
+      </c>
+      <c r="U26" t="inlineStr">
+        <is>
+          <t>DNF</t>
+        </is>
+      </c>
+      <c r="V26" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -1492,6 +1817,20 @@
       <c r="P27" t="n">
         <v>2</v>
       </c>
+      <c r="S27" t="n">
+        <v>22</v>
+      </c>
+      <c r="T27" t="inlineStr">
+        <is>
+          <t>Tudge Boat</t>
+        </is>
+      </c>
+      <c r="U27" t="n">
+        <v>21.73263</v>
+      </c>
+      <c r="V27" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -1538,6 +1877,20 @@
       <c r="P28" t="n">
         <v>2</v>
       </c>
+      <c r="S28" t="n">
+        <v>23</v>
+      </c>
+      <c r="T28" t="inlineStr">
+        <is>
+          <t>dtmittens</t>
+        </is>
+      </c>
+      <c r="U28" t="n">
+        <v>21.79796</v>
+      </c>
+      <c r="V28" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -1586,6 +1939,20 @@
       <c r="P29" t="n">
         <v>1</v>
       </c>
+      <c r="S29" t="n">
+        <v>24</v>
+      </c>
+      <c r="T29" t="inlineStr">
+        <is>
+          <t>timesprout</t>
+        </is>
+      </c>
+      <c r="U29" t="n">
+        <v>22.12472</v>
+      </c>
+      <c r="V29" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -1630,6 +1997,20 @@
       <c r="P30" t="n">
         <v>1</v>
       </c>
+      <c r="S30" t="n">
+        <v>25</v>
+      </c>
+      <c r="T30" t="inlineStr">
+        <is>
+          <t>Waaksaam</t>
+        </is>
+      </c>
+      <c r="U30" t="n">
+        <v>22.34469</v>
+      </c>
+      <c r="V30" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -1662,6 +2043,20 @@
       <c r="J31" t="n">
         <v>2</v>
       </c>
+      <c r="S31" t="n">
+        <v>26</v>
+      </c>
+      <c r="T31" t="inlineStr">
+        <is>
+          <t>Noxitu</t>
+        </is>
+      </c>
+      <c r="U31" t="n">
+        <v>22.39215</v>
+      </c>
+      <c r="V31" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -1694,6 +2089,20 @@
       <c r="J32" t="n">
         <v>2</v>
       </c>
+      <c r="S32" t="n">
+        <v>27</v>
+      </c>
+      <c r="T32" t="inlineStr">
+        <is>
+          <t>[CSC]IronDragon111000</t>
+        </is>
+      </c>
+      <c r="U32" t="n">
+        <v>22.50038</v>
+      </c>
+      <c r="V32" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -1726,6 +2135,20 @@
       <c r="J33" t="n">
         <v>2</v>
       </c>
+      <c r="S33" t="n">
+        <v>28</v>
+      </c>
+      <c r="T33" t="inlineStr">
+        <is>
+          <t>pannekoekbijter</t>
+        </is>
+      </c>
+      <c r="U33" t="n">
+        <v>22.63835</v>
+      </c>
+      <c r="V33" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -1758,6 +2181,22 @@
       <c r="J34" t="n">
         <v>2</v>
       </c>
+      <c r="S34" t="n">
+        <v>29</v>
+      </c>
+      <c r="T34" t="inlineStr">
+        <is>
+          <t>PlusMicron</t>
+        </is>
+      </c>
+      <c r="U34" t="inlineStr">
+        <is>
+          <t>DNF</t>
+        </is>
+      </c>
+      <c r="V34" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -1790,6 +2229,22 @@
       <c r="J35" t="n">
         <v>1</v>
       </c>
+      <c r="S35" t="n">
+        <v>29</v>
+      </c>
+      <c r="T35" t="inlineStr">
+        <is>
+          <t>[CCC]Shinikage221</t>
+        </is>
+      </c>
+      <c r="U35" t="inlineStr">
+        <is>
+          <t>DNF</t>
+        </is>
+      </c>
+      <c r="V35" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -1822,6 +2277,20 @@
       <c r="J36" t="n">
         <v>1</v>
       </c>
+      <c r="S36" t="n">
+        <v>31</v>
+      </c>
+      <c r="T36" t="inlineStr">
+        <is>
+          <t>[Buny]Lunarbunny</t>
+        </is>
+      </c>
+      <c r="U36" t="n">
+        <v>25.19011</v>
+      </c>
+      <c r="V36" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -1838,6 +2307,20 @@
       <c r="D37" t="n">
         <v>3</v>
       </c>
+      <c r="S37" t="n">
+        <v>32</v>
+      </c>
+      <c r="T37" t="inlineStr">
+        <is>
+          <t>Orb Bee Bob</t>
+        </is>
+      </c>
+      <c r="U37" t="n">
+        <v>25.33275</v>
+      </c>
+      <c r="V37" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -1854,6 +2337,20 @@
       <c r="D38" t="n">
         <v>3</v>
       </c>
+      <c r="S38" t="n">
+        <v>33</v>
+      </c>
+      <c r="T38" t="inlineStr">
+        <is>
+          <t>[SLOW]Zeus</t>
+        </is>
+      </c>
+      <c r="U38" t="n">
+        <v>26.25868</v>
+      </c>
+      <c r="V38" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -1870,6 +2367,20 @@
       <c r="D39" t="n">
         <v>2</v>
       </c>
+      <c r="S39" t="n">
+        <v>34</v>
+      </c>
+      <c r="T39" t="inlineStr">
+        <is>
+          <t>SuperHeavy</t>
+        </is>
+      </c>
+      <c r="U39" t="n">
+        <v>23.25999</v>
+      </c>
+      <c r="V39" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -1885,6 +2396,22 @@
       </c>
       <c r="D40" t="n">
         <v>2</v>
+      </c>
+      <c r="S40" t="n">
+        <v>35</v>
+      </c>
+      <c r="T40" t="inlineStr">
+        <is>
+          <t>CaptainD54321 (they/she)</t>
+        </is>
+      </c>
+      <c r="U40" t="inlineStr">
+        <is>
+          <t>DNF</t>
+        </is>
+      </c>
+      <c r="V40" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="41">

</xml_diff>

<commit_message>
Troll 4: exclude aizpun (joined briefly, did not compete)
aizpun was registered in the lobby and the game logged a R1 DNF, but
user did not actually play this cup. 29 ranked players now (was 30).
Score unchanged (aizpun was at pos 23 with 0 pts; everyone else's
finish position unchanged since they were above aizpun).

Also fixes add_cup50.py clear loop: ws.cell(row, col, value=None) does
NOT clear existing cell content in openpyxl — only initializes empty
cells. Use ws.cell(row, col).value = None instead. Previous run had
left aizpun stranded at row 35 even after EXCLUDE was set.
Same bug pattern exists in add_cup46-49.py if re-run.
</commit_message>
<xml_diff>
--- a/Petite Cups 46-50.xlsx
+++ b/Petite Cups 46-50.xlsx
@@ -2724,22 +2724,6 @@
       <c r="V35" t="n">
         <v>3</v>
       </c>
-      <c r="Y35" t="n">
-        <v>23</v>
-      </c>
-      <c r="Z35" t="inlineStr">
-        <is>
-          <t>aizpun</t>
-        </is>
-      </c>
-      <c r="AA35" t="inlineStr">
-        <is>
-          <t>DNF</t>
-        </is>
-      </c>
-      <c r="AB35" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="36">
       <c r="A36" t="n">

</xml_diff>